<commit_message>
feat: add goal management features with CRUD operations and notification enhancements
</commit_message>
<xml_diff>
--- a/requirement-plan.xlsx
+++ b/requirement-plan.xlsx
@@ -58,7 +58,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,7 +74,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -82,6 +82,12 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -141,25 +147,25 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -474,20 +480,20 @@
   <cols>
     <col min="1" max="1" style="10" width="28.14785714285714" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="11" width="62.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="30.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -523,7 +529,7 @@
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="7">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -542,11 +548,11 @@
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="58.5">
-      <c r="A4" s="7" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="60.75">
+      <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="6"/>
@@ -561,11 +567,11 @@
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="72" customFormat="1" s="9">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="75" customFormat="1" s="7">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="5"/>
@@ -580,7 +586,7 @@
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="7">
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
@@ -597,7 +603,7 @@
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" customFormat="1" s="7">
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
@@ -614,7 +620,7 @@
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="7">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>

</xml_diff>